<commit_message>
feat: sync updated Donguibogam headache matrix (15 patterns/20 acupoints) and replace portal web documents
</commit_message>
<xml_diff>
--- a/04_번역원고_및_임상매트릭스/오십견_누견풍_침구해부_매트릭스/오십견_누견풍_해부임상_매트릭스.xlsx
+++ b/04_번역원고_및_임상매트릭스/오십견_누견풍_침구해부_매트릭스/오십견_누견풍_해부임상_매트릭스.xlsx
@@ -16,6 +16,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_조구투승산_고증계보" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_생의학_신경반사_LayerA_B" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_ARI_v3_평가표" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제1_FMA특징" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제2_유사도" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제3_운동기능해부" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제4_3D측정" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제5_인용검증" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제6_이력" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="정제7_지침검증" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +51,15 @@
       <color rgb="00334155"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +96,16 @@
         <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008E44AD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -109,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -128,6 +152,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1010,6 +1043,3667 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>코드</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>혈명</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>분절</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>어깨관절 지배신경</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>더부신경</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>신경 영역</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>FMA 구조 수</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>다분절 제외</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Axillary nerve, Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Anterior branch of axillary nerve; Axillary nerve; Inferior lateral cutaneous nerve of arm; Musculocutaneous nerve; Peripheral segment of musculocutaneous nerve; Peripheral segment of radial nerve; Posterior branch of axillary nerve; Superior subscapular nerve; Supraclavicular nerve; Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Axillary nerve, Set of muscular branches of axillary nerve, Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Anterior branch of axillary nerve; Axillary nerve; Lateral supraclavicular nerve; Posterior branch of axillary nerve; Set of muscular branches of axillary nerve; Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>C5,C6,C7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Axillary nerve, Lateral pectoral nerve</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Axillary nerve; Lateral pectoral nerve; Musculocutaneous nerve</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>C5,C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Axillary nerve</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Anterior branch of axillary nerve; Axillary nerve; Inferior subscapular nerve; Peripheral segment of radial nerve; Posterior branch of axillary nerve; Radial nerve; Superior lateral cutaneous nerve of arm; Thoracodorsal nerve</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Axillary nerve, Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Anterior branch of axillary nerve; Axillary nerve; Inferior subscapular nerve; Lateral supraclavicular nerve; Peripheral segment of radial nerve; Posterior branch of axillary nerve; Radial nerve; Superior lateral cutaneous nerve of arm; Suprascapular nerve; Thoracodorsal nerve</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6,C7,C8</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Axillary nerve, Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Anterior branch of axillary nerve; Axillary nerve; Inferior subscapular nerve; Lateral supraclavicular nerve; Posterior branch of axillary nerve; Suprascapular nerve; Thoracodorsal nerve</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LI16</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>巨骨</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Anterior ramus of fourth cervical nerve; Anterior ramus of third cervical nerve; Lateral supraclavicular nerve; Spinal accessory nerve; Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6,C7,C8,T1,T2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Lateral pectoral nerve</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Brachial nerve plexus; Cervical branch of facial nerve; Facial nerve; Intermediate supraclavicular nerve; Lateral pectoral nerve; Long thoracic nerve; Medial pectoral nerve; Peripheral segment of supraclavicular nerve; Second intercostal nerve; Supraclavicular nerve</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GB21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>肩井</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>C3,C4,C5,C6</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Anterior ramus of fifth cervical nerve; Anterior ramus of fourth cervical nerve; Anterior ramus of third cervical nerve; Dorsal scapular nerve; Fifth cervical nerve; Spinal accessory nerve; Supraclavicular nerve; Suprascapular nerve</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Splenius cervicis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ST38</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>條口</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>L3,L4,L5,S1,S2,S3,S4</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Common fibular nerve; Deep fibular nerve; Medial terminal branch of deep fibular nerve; Sacral nerve plexus; Sciatic nerve; Set of medial crural cutaneous branches of saphenous nerve; Superficial fibular nerve</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BL57</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>承山</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>L4,L5,S1,S2,S3,S4</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Common fibular nerve; Lateral sural cutaneous nerve; Medial sural cutaneous nerve; Posterior femoral cutaneous nerve; Sacral nerve plexus; Sciatic nerve; Tibial nerve</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TE3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>中渚</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>C5,C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Deep branch of ulnar nerve; Peripheral segment of ulnar nerve; Posterior interosseous nerve; Radial nerve</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LI11</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>曲池</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>C5,C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Inferior lateral cutaneous nerve of arm; Lateral cutaneous nerve of forearm; Peripheral segment of musculocutaneous nerve; Peripheral segment of radial nerve; Posterior cutaneous nerve of forearm; Posterior interosseous nerve; Radial nerve; Superficial branch of radial nerve</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LI4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>合谷</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>C6,C7,C8,T1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Deep branch of ulnar nerve; Peripheral segment of ulnar nerve; Set of dorsal digital branches of radial nerve</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GB34</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>陽陵泉</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>L4,L5,S1,S2,S3,S4</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Common fibular nerve; Deep fibular nerve; Medial terminal branch of deep fibular nerve; Sacral nerve plexus; Sciatic nerve; Superficial fibular nerve</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr"/>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>LI16</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>GB21</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>ST38</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>BL57</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>TE3</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t>LI11</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>LI4</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t>GB34</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.319</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.387</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LI16</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.601</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GB21</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.601</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ST38</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BL57</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.446</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TE3</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.214</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.489</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LI11</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.319</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.248</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LI4</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.489</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.248</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GB34</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>운동</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>코드</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>혈명</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>주동근(A)</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>제한 근육(R)</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>원 보고서 배정</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>관절낭 제한(B1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Subscapularis</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Teres minor, Infraspinatus</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Infraspinatus</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Infraspinatus, Teres minor</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ER 외회전</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대·위/중간 오목위팔인대(rotator interval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Subscapularis</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Teres minor, Infraspinatus</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Infraspinatus</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Infraspinatus, Teres minor</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IR 내회전</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Deltoid, Coracobrachialis, Short head of biceps brachii, Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi, Long head of triceps brachii</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Long head of triceps brachii, Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>FL 굽힘(전방거상)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·뒤 관절낭</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Deltoid, Supraspinatus</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>LI16</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>巨骨</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Supraspinatus</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AB 벌림(외전)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>GB21</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>肩井</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Supraspinatus</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>아래 관절낭(겨드랑오목)·아래 오목위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>LI15</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>肩髃</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TE14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>肩髎</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EX-UE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>肩前</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Deltoid</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Coracobrachialis, Short head of biceps brachii, Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SI9</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>肩貞</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Deltoid, Teres major, Latissimus dorsi, Long head of triceps brachii</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SI10</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>臑俞</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Deltoid, Long head of triceps brachii, Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SI11</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>天宗</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Deltoid, Teres major, Latissimus dorsi</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EX 폄(후방신전)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LU2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>雲門</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pectoralis major</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>앞 관절낭·부리위팔인대</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>구조/혈</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>FMA</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>부피(cm³)</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>크기·거리</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>닫힘</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Supraspinatus</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9629</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.65</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>125×79×35</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Infraspinatus</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>32546</v>
+      </c>
+      <c r="C3" t="n">
+        <v>106.28</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>129×81×124</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Subscapularis</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>13413</v>
+      </c>
+      <c r="C4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>103×97×130</t>
+        </is>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Teres minor</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>32550</v>
+      </c>
+      <c r="C5" t="n">
+        <v>32.78</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>85×68×96</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Teres major</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>32549</v>
+      </c>
+      <c r="C6" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>86×81×96</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LI16 巨骨 — Supraspinatus</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9629</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 50.47 mm / 둘째갈비뼈 25.83 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GB21 肩井 — Levator scapulae</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>32519</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 13.24 mm / 둘째갈비뼈 13.03 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GB21 肩井 — Supraspinatus</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9629</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 50.47 mm / 둘째갈비뼈 25.79 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GB21 肩井 — Descending part of right trapezius</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>33586</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 9.75 mm / 둘째갈비뼈 12.71 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LU2 雲門 — Subclavius</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>13410</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 0.05 mm / 둘째갈비뼈 2.99 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LU2 雲門 — Pectoralis minor</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>13109</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 45.4 mm / 둘째갈비뼈 13.35 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LU2 雲門 — Right pectoralis major</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>13373</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 13.26 mm / 둘째갈비뼈 0.15 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SI11 天宗 — Infraspinatus</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>32546</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 75.85 mm / 둘째갈비뼈 50.99 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LI15 肩髃 — Supraspinatus</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>9629</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 50.51 mm / 둘째갈비뼈 25.87 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LI15 肩髃 — Subscapularis</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>13413</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>첫째갈비뼈 46.51 mm / 둘째갈비뼈 17.16 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>폐 메쉬(7309·7333)는 기관지 나무뿐 — 흉막·폐 표면 거리 측정 불가, 갈비뼈는 대리 지표</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>인용</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>실제</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PMID 23620934 = papers.id 1836</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>中国针灸 2013 — 경혈 마사지 &gt; 전침·TENS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>기전 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>papers.id 397</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>J Pain Res 2023 — 침도 후향 연구</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>기전 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PMID 17333364</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>J Assist Reprod Genet 2007 — 자궁내막증 마이크로어레이</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>무관(잘못된 PMID)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PMID 25069201</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>针刺研究 2014 — 뇌졸중 어깨-손 증후군 外關 온침</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>天宗 GTO 기전과 무관</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PMID 32952592 = papers.id 1819</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>eCAM 2020 — 건강 여성 근지구력 예비 연구</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>雲門 기전과 무관</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>papers.id 1827</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>中国针灸 2026 — 天府 어깨 주치 교재 고찰</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>雲門 기전 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9절 SMD −0.85</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>출처 없음</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cochrane 2005(PMID 15846753): 근거 부족·단기 이득 가능성</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>《逢源》 肩節如膠</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>证治通鉴_21 L1303(《针灸逢源·症治要穴歌》 표제)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>출전 표기 확정·원천 미확정(허임 《鍼灸經驗方》 대조 필요)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>條口 계보</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>针灸腧穴通考_08 L1131~1153</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>일치(왕문면→王文綿)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>《席弘賦》·《世醫得效方》·《類經圖翼》</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>证治通鉴_21 L1043·L1213·L1221·L1263</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>일치</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>《玉龍歌》 肩端紅腫</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>证治通鉴_21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>92% 일치(중간 생략)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>일자</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>작업</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>도구</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>최초 작성</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FMA 분석·이미지 추가, 인용·운동학·Layer A·ARI 감사</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>문헌</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>PMID</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>확인 범위</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>침 치료 취급</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>핵심 원문</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Kelley 2013 JOSPT CPG (APTA)</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>23636125</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>10.2519/jospt.2013.0302</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>전문 PDF</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>권고 없음(전침 RCT 1건 근거 서술에만 인용)</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>신장 운동: 조직 과민성에 따라 강도(B); 스테로이드+운동&gt;운동(A); 기기: 단파·초음파·전기자극(C)</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>검토 의견 맞음</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Rupani·Gwilym 2025 BESS pathway</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>40291049</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>10.1177/17585732251335955</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>PMC 전문</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>언급 0회</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>GRADE 11 PICO: 물리치료·스테로이드·수압팽창·MUA·관절낭 유리술</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>검토 의견 맞음</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>NICE CKS frozen shoulder</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>2차 인용(PMC10909438)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>2차 문헌에 언급 없음</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>일차 진료: 진통제·물리치료·관절 주사 조기 관리</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>부분 확인(원문 대조 필요)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Ewald 2011 Am Fam Physician</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>21322517</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>전문</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>비권고(추가 연구 필요, B)</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Acupuncture may be helpful … further study is needed before it can be recommended</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>검토 의견 맞음</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Green 2005 Cochrane CD005319</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>15846753</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>10.1002/14651858.CD005319</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>전문</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>근거 부족·단기 이득 가능성</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Sun 2001(PMID 11773673): 침+운동&gt;운동, WMD 9.20/9.40(20주)</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>검토 의견 맞음</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Ben-Arie 2020 eCAM SR/MA</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>33062030</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>10.1155/2020/9790470</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>PMC 전문</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>개인 종설 의견(Jain 등 "중등도 권고") 소개, 학회 지침 아님</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>VAS·CMS·굴곡 우세, 근거 수준 매우 낮음</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>검토 의견 맞음</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>견비통 한의표준임상진료지침 2020 (G-KoM/한국한의약진흥원, ISBN 979-11-5955-547-3)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>원문 PDF 208쪽</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>R3 침+자가운동 B/Moderate; R4 침+물리치료 A/High; R9 동기침법·R10 조구-승산 심자·R12 조구 전침 C/Low</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>적용 범위 = 견비통 전반(M75.0 포함), 질환별 하위 권고 없음. 운동 단독 권고는 근거 부족으로 미도출</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>국내 한의 지침은 병행 권고함(견비통 전반)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Johansson 2005 Phys Ther (KCPG R3 근거)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>15921471</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>침+자가운동 vs 초음파+자가운동</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>충격증후군 85명; 12개월째만 유의</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>동결견 직접 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Johansson 2011 Fam Pract (KCPG R3 근거)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>21378086</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>10.1093/fampra/cmq119</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>침+자가운동 vs 스테로이드 주사</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>충격증후군 91명; 모든 시점 유의차 없음</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>동결견 직접 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Vas 2008 Rheumatology (KCPG R4·R9 근거)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>18403402</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>10.1093/rheumatology/ken040</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>단일혈 침+물리치료 vs mock TENS+물리치료</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>견봉하 증후군 425명; CMS +6.0점; KCPG 본문은 대조군을 "경피신경전기자극"으로 표기</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>동결견 직접 근거 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Sun 2001 Hong Kong Med J</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>11773673</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>침+운동 vs 운동</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>동결견 35명; 6주·20주 유의. KCPG 본문은 대조군을 "대기지연치료/거짓 침"으로 오기</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>동결견 유일 직접 병행 근거</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>결론</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>국제 지침: 침 비권고(9절 4항 정정). 국내 KCPG: 견비통 전반에 침+운동(B)·침+물리치료(A) 권고, 근거는 충격증후군 RCT. 보고서 9.1·9.2절</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>정정·보완 완료</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>